<commit_message>
new updates in paper
</commit_message>
<xml_diff>
--- a/frontend/public/sample_file/paragraph_questions_upload_template.xlsx
+++ b/frontend/public/sample_file/paragraph_questions_upload_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paragraph_Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Paragraph Questions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,23 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +56,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,252 +429,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>classId</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>subjectId</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>topicId</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>question_type</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>paragraph_group_id</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>instruction_text</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>paragraph</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sub_question_id</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>sub_question_type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>sub_question_text</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>option_A</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>option_B</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>option_C</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>option_D</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>correct_answer</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>marks</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>negative_marks</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>class_10</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>physics</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>science</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>environmental_science</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>paragraph</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Read the following passage carefully and answer the questions that follow.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Here is a paragraph about the Solar System...</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>SQ1</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>mcq_text</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Which celestial body holds most of the Solar System's mass?</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jupiter</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>The Sun</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Earth</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Moon</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Study the water cycle passage and answer the following questions.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>The water cycle is the continuous process of water moving from Earth's surface to the atmosphere and back. It consists of four main stages: evaporation, condensation, precipitation, and collection. Evaporation occurs when water from oceans, lakes, and rivers turns into water vapor due to heat from the sun. Condensation is when water vapor cools and forms clouds. Precipitation is when water falls back to Earth as rain, snow, or hail. Finally, collection occurs when water gathers in oceans and lakes.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>What is the first stage of the water cycle?</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Condensation</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Evaporation</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Precipitation</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>class_10</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>physics</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>science</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>environmental_science</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Study the water cycle passage and answer the following questions.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>The water cycle is the continuous process of water moving from Earth's surface to the atmosphere and back. It consists of four main stages: evaporation, condensation, precipitation, and collection. Evaporation occurs when water from oceans, lakes, and rivers turns into water vapor due to heat from the sun. Condensation is when water vapor cools and forms clouds. Precipitation is when water falls back to Earth as rain, snow, or hail. Finally, collection occurs when water gathers in oceans and lakes.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Which process occurs when water vapor cools?</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Evaporation</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Condensation</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Collection</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Precipitation</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>science</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>environmental_science</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Study the water cycle passage and answer the following questions.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>The water cycle is the continuous process of water moving from Earth's surface to the atmosphere and back. It consists of four main stages: evaporation, condensation, precipitation, and collection. Evaporation occurs when water from oceans, lakes, and rivers turns into water vapor due to heat from the sun. Condensation is when water vapor cools and forms clouds. Precipitation is when water falls back to Earth as rain, snow, or hail. Finally, collection occurs when water gathers in oceans and lakes.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>true_false</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Precipitation is when water falls back to Earth.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>reading</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>paragraph</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Read the following passage carefully and answer the questions that follow.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Here is a paragraph about the Solar System...</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>SQ2</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>mcq_text</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>What are the inner planets mainly made of?</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Gas and Ice</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Liquid Water</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Rock and Metal</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Dust and Helium</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Read the following excerpt and answer the questions.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>The Industrial Revolution marked a major turning point in human history. Beginning in Britain in the late 1700s, it transformed agrarian societies into industrial ones. Key inventions like the steam engine and textile machinery powered economic growth and urbanization.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>When did the Industrial Revolution begin?</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Early 1600s</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Late 1700s</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Early 1800s</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Mid 1800s</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>reading</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>paragraph</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Read the following excerpt and answer the questions.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>The Industrial Revolution marked a major turning point in human history. Beginning in Britain in the late 1700s, it transformed agrarian societies into industrial ones. Key inventions like the steam engine and textile machinery powered economic growth and urbanization.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>short_answer</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Name one key invention of the Industrial Revolution.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>steam engine</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>